<commit_message>
Add excel_style.py for consistent Excel formatting across reports
</commit_message>
<xml_diff>
--- a/battlebots_2015_2025.xlsx
+++ b/battlebots_2015_2025.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season 11 (2021)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season 12 (2022)" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Features" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Correlations" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20002,7 +20003,6 @@
           <t>2x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20043,13 +20043,6 @@
           <t>Flipper</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -20057,8 +20050,6 @@
           <t>Axe Backwards</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20074,7 +20065,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Team Axe Backwards (formerly KurTrox Robotix)</t>
@@ -20095,13 +20085,6 @@
           <t>Full body drum spinner</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -20114,7 +20097,6 @@
           <t>2x Long Magmotors</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>235lbs</t>
@@ -20165,11 +20147,6 @@
           <t>6x MaxAmps 3S LiPo batteries</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -20182,7 +20159,6 @@
           <t>2x Long Magmotors</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>227lbs (WC III) [ 1 ]</t>
@@ -20198,7 +20174,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Forge &amp; Farm Combat Robots</t>
@@ -20224,12 +20199,6 @@
           <t>Blacksmith (Kyle Singer, Earl Pancoast III) Red Devil (Earl Pancoast III) Animosity (Alex Grant) The Executioner , Roadkill (Miro Matheson)</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -20242,7 +20211,6 @@
           <t>4x Flipsky 6384 brushless motors</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20258,7 +20226,6 @@
           <t>BattleBots: Champions II BattleBots Pro League (2026) (Alternate)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Team Small Robots</t>
@@ -20294,10 +20261,6 @@
           <t>BattleBots Proving Ground (2023) BattleBots Proving Ground (2024) BattleBots FaceOffs (2025)</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -20305,8 +20268,6 @@
           <t>Basilisk</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>245lbs</t>
@@ -20317,8 +20278,6 @@
           <t>World Championship II World Championship III</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>MBS Robotics</t>
@@ -20339,13 +20298,6 @@
           <t>Flipper Pneumatic spike (WC II) Flamethrower (WC III)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -20358,14 +20310,11 @@
           <t>2x Electric scooter motors</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>World Championship III</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Bacon Double Slamburger (Working name)</t>
@@ -20401,15 +20350,11 @@
           <t>8S LiPo batteries</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>Gloomweaver , Fowl Play</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -20417,8 +20362,6 @@
           <t>BattleSaw</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20429,8 +20372,6 @@
           <t>World Championship II (Not selected) World Championship III (Withdrew) World Championship IV World Championship V (Withdrew)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Twister Robotics</t>
@@ -20456,12 +20397,6 @@
           <t>Gamma 9 , Namreko 3000 , Gammatron , Gammacide (Curtis Nemeth) Bellator , Swamp Thing (Mark Elam)</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -20474,7 +20409,6 @@
           <t>2x Maytech 6880 brushless motors (WC VII-Present) 2x 48v Bosch DC motors (WC I-BB: Bounty Hunters) 2x 36V Magmotor S28-200 motors (Season 5.0)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>250lbs (WC I-Present) 219lbs (Season 5.0)</t>
@@ -20525,7 +20459,6 @@
           <t>12S LiPo batteries 3Ah NiCad BattlePacks (Season 5.0)</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>KillerHurtz , TerrorHurtz</t>
@@ -20536,8 +20469,6 @@
           <t>Season 5.0 (Withdrew)</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -20550,7 +20481,6 @@
           <t>4x Maytech 6374 brushless motors</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20596,16 +20526,11 @@
           <t>WAR Hawk , Jäger (Emmanuel Carrillo, Andy Russell) Overhaul (Elizabeth Cao) Horizon (Tommy Wong) MadCatter (Emmanuel Carrillo, Ryan Lau) Malice (Isaak Malers) Chronos (Trent Wilson) Dark Steel , Dark Shredder , Dome of Darkness (Russ Barrow) Goblin (Ellis Ware)</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -20618,7 +20543,6 @@
           <t>2x S28-400 Magmotors (9hp) [ 2 ]</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20669,15 +20593,11 @@
           <t>10x 5Ah 6S Turnigy Nano-tech LiPo batteries (WC II-WC III) [ 1 ]</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
           <t>Brutality , Green Wave , Tantrum , Ntertainment , Land Shark , Knockturnal</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -20690,7 +20610,6 @@
           <t>2x 8025 Brushless motors (WCVIII-Present) 2x Magmotors (WC IV-BB: Champions II)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20706,7 +20625,6 @@
           <t>BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Team Uai!rrior</t>
@@ -20727,13 +20645,6 @@
           <t>Eggbeater drum spinner Flamethrower</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -20741,9 +20652,6 @@
           <t>Black Widow</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>World Championship V</t>
@@ -20754,7 +20662,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Team Black Widow</t>
@@ -20775,13 +20682,6 @@
           <t>Drum spinner Flamethrower</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -20789,8 +20689,6 @@
           <t>Blacksmith</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20806,7 +20704,6 @@
           <t>BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Team Half Fast Astronaut</t>
@@ -20832,12 +20729,6 @@
           <t>Bale Spear (Earl Pancoast III, Kyle Singer) Golem , Scuttle (James Iocca)</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -20850,7 +20741,6 @@
           <t>2x TP5680 brushless motors</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -20896,16 +20786,11 @@
           <t>Insult and Injury (Aren Hill, Jason Weihman, Bryan Culver)</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>Tantrum , The Twins</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -20918,7 +20803,6 @@
           <t>4x Brushless TP Motors</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>247-250lbs</t>
@@ -20979,9 +20863,6 @@
           <t>Retrograde , Subatomic , Fireball</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -20994,7 +20875,6 @@
           <t>4x Magmotors</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>245-250lbs</t>
@@ -21005,8 +20885,6 @@
           <t>World Championship II World Championship III World Championship IV</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Chaos Corps</t>
@@ -21037,11 +20915,6 @@
           <t>8s 10Ah LiPo battery</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -21054,7 +20927,6 @@
           <t>4x Magmotors</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>140lbs (Cisco Party 2006) 220lbs (2009, WC IV)</t>
@@ -21070,7 +20942,6 @@
           <t>Cisco Party 2006</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Team Nightmare</t>
@@ -21091,25 +20962,21 @@
           <t>Lifting scoop Hammer (WC IV)</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>MaxAmps LiPo batteries</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
           <t>Rhino , Junior , Nightmare , Backlash , Whirligig , Turtle , ShazBot , MicroNightmare , Wallop , Grasshopper , The Swarm ( Locust )</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr">
         <is>
           <t>Pro Championship 2009</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -21122,7 +20989,6 @@
           <t>6x 3" Brushed motors (WC II) 4x motors (WC I, WC III-Present)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -21138,7 +21004,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2019) BattleBots: Bounty Hunters BattleBots: Destruct-A-Thon</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Inertia Labs</t>
@@ -21159,21 +21024,16 @@
           <t>Flipping arm</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>LiFePO batteries (Destruct-A-Thon)</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
           <t>Toro , The Matador , T-Minus , Rhino , The Butcher</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -21186,7 +21046,6 @@
           <t>2x Brushless motors (WC III) 2x NPC brushed motors (WC II)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>242lbs</t>
@@ -21197,8 +21056,6 @@
           <t>World Championship II World Championship III</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Team Brutus</t>
@@ -21224,12 +21081,6 @@
           <t>Overhaul , Witch Doctor , Coincidence (Adam Bercu) Valkyrie , RIPperoni , Starchild (Amanda Fowler)</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -21237,8 +21088,6 @@
           <t>Captain Shrederator</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>220lbs [ 1 ]</t>
@@ -21284,16 +21133,11 @@
           <t>Lucky (Zac O'Donnell) Raven , Ultimo Destructo , Purple Fire (Jacob Rogers) Skorpios , Malice (Jonathan LaPlain) Triton , Deep Six , Bad Kitty , Switchback , Chronos , VD6.0 (Bradley Hanstad)</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
           <t>Chopper , Code:BLACK , Dispose-All , Phrizbee , Phrizbee-Ultimate , Shredhead , Pincer</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -21301,8 +21145,6 @@
           <t>Chomp</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>250lbs (WC I-re:MARS 2019) 500lbs (WC V-BB: Bounty Hunters)</t>
@@ -21318,7 +21160,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2019) BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>The Machine Corps</t>
@@ -21344,12 +21185,6 @@
           <t>The Judge , The Prosecutor , Juggernaut (Jascha Little)</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -21357,8 +21192,6 @@
           <t>Chronos</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>243lbs</t>
@@ -21374,7 +21207,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Team Chronos</t>
@@ -21405,15 +21237,11 @@
           <t>MaxAmps LiPo batteries</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
           <t>No Luv , El Cucuy</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -21426,7 +21254,6 @@
           <t>4x RV-120E brushless motors</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>250lbs ~238lbs (WC V) [ 1 ]</t>
@@ -21472,16 +21299,11 @@
           <t>WAR Hawk (Kevin Milczewski, Joshua Beavers)</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>BattleBots Proving Ground BattleBots FaceOffs (2024)</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -21494,8 +21316,6 @@
           <t>2x HyperDrive motors</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>World Championship II World Championship IV World Championship V (Withdrew) World Championship VI World Championship VII</t>
@@ -21506,7 +21326,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2022) BattleBots: Champions II BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Robotic Death Company (WC VI-Present) Team Carbide (WC II, WC IV)</t>
@@ -21532,7 +21351,6 @@
           <t>Axolotl , Horizon (Alon Belkin) Wrecks , Skorpios , Tiki Fire (Micah Leibowitz) Stinger: The Killer Bee , Devil's Plunger , Sewer Snake , Wipe Out #2 (Matt Maxham, Wendy Maxham) Quantum (James Cooper) Beta (Dave Moulds) Taco Tuesday (Camden Wallraff) Lucky (Matt Olson, Mark Demers) Calypso (Alon Belkin, Derek Tran, Alex Price) Manta , Golden Fury (Derek Tran) JackPot (Derek Tran, David Le) Banshee (Alon Belkin, Alex Price) Nemesis (David Le) Ziggy , CycloneBot , PitBot , BravePart (Mark Demers)</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs (2024)</t>
@@ -21543,9 +21361,6 @@
           <t>Gigabyte , Megabyte , Rambite , Invader , Super Megabyte , Agsma</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -21558,7 +21373,6 @@
           <t>2x Maytech MTO6365 motors (BB Pro League 2026)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -21609,15 +21423,11 @@
           <t>5Ah 6S LiPo batteries</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>Poison Arrow</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -21630,7 +21440,6 @@
           <t>4x Maytech 65162 brushless motors</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -21681,15 +21490,11 @@
           <t>4x MaxAmps 4Ah 37V 150C LiPo batteries</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
           <t>The Ringmaster , Marvin</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -21702,14 +21507,11 @@
           <t>2x Custom motors</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>World Championship IV</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>Daisycutter</t>
@@ -21735,17 +21537,11 @@
           <t>Vertical spinning disks</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -21758,7 +21554,6 @@
           <t>T-MOTOR P80III KV100 motors</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -21774,7 +21569,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>RoboGym Robotics</t>
@@ -21795,17 +21589,11 @@
           <t>Lifter Grappler (WC VI-BB: Champions I) Flamethrower</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
           <t>Roundhouse , Snatch</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -21813,8 +21601,6 @@
           <t>DeathRoll</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>243-250lbs</t>
@@ -21855,17 +21641,11 @@
           <t>Vertical spinning disk</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>48V LiPo battery system</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -21878,7 +21658,6 @@
           <t>2x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -21894,7 +21673,6 @@
           <t>BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>Team Overboard</t>
@@ -21925,15 +21703,11 @@
           <t>3.4Ah 6S LiPo batteries</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
           <t>Triton</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -21946,7 +21720,6 @@
           <t>4x Magmotors</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -21962,7 +21735,6 @@
           <t>BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>Team Fast Electric Robots</t>
@@ -21988,16 +21760,11 @@
           <t>Bite Force , Lucky , Scrap Metal , FrostBite (Rob Masek) Manta (Matt Vasquez) Valkyrie (Jason Vasquez) VD6.0 (Jeff Vasquez)</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
           <t>Whiplash , Splatter , Deb Bot , Matts Bammer , Think Tank</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -22005,8 +21772,6 @@
           <t>Deviled Egg</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22017,8 +21782,6 @@
           <t>World Championship III World Championship VI (Not selected)</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>Recoil Robotics</t>
@@ -22044,12 +21807,6 @@
           <t>Sharko , Riptide (Zak Hassanein) Mega Tento (Ryan Hasty) Clockwork L'Orange (Shannon &amp; Kathy O'Hare)</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -22057,12 +21814,6 @@
           <t>Doom</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>Team Bad Bot</t>
@@ -22083,17 +21834,11 @@
           <t>Hinged wedge</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr">
         <is>
           <t>NPC Charity Open</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -22106,7 +21851,6 @@
           <t>2x Surpass 70120 brushless motors</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22117,7 +21861,6 @@
           <t>World Championship VII (Alternate)</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>Dooomba</t>
@@ -22148,12 +21891,6 @@
           <t>Battle Royale With Cheese (Brice Farrell) Mammoth (Thuong Nguyen, Brice Farrell, Liz Chavarria) Sporkinok (Liz Chavarria) Pardon My French (Philippe Voyer)</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -22166,7 +21903,6 @@
           <t>4x Long Magmotors</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>248½lbs</t>
@@ -22177,8 +21913,6 @@
           <t>World Championship II (Withdrew) World Championship III</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>Iron LungFish Robotics</t>
@@ -22199,17 +21933,11 @@
           <t>Twin horizontal bar spinners</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
           <t>Chomp . Mongus , Spwack</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -22222,7 +21950,6 @@
           <t>2x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>248lbs</t>
@@ -22263,17 +21990,11 @@
           <t>Cannon</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>8Ah 25C LiPo battery</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -22281,8 +22002,6 @@
           <t>Double Tap</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22293,7 +22012,6 @@
           <t>World Championship VII (Alternate) BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>DoubleTap</t>
@@ -22319,13 +22037,6 @@
           <t>Adjustable angled blade with centrifical hammers</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -22333,16 +22044,11 @@
           <t>Dragon King</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>World Championship VII (Alternate)</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Bots Bash Party Crew</t>
@@ -22368,7 +22074,6 @@
           <t>Slap 'Em Silly Slap 'Em Sillier Sledge-Jammer (Andy Sauro) Tombstone (Zach Lytle)</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>BattleBots Proving Ground (2026)</t>
@@ -22379,9 +22084,6 @@
           <t>Skorpios</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -22394,7 +22096,6 @@
           <t>2x Long Magmotors (WC VII-Present) 2x NPC-T64 motors (WC VI)</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>225-250lbs</t>
@@ -22445,15 +22146,11 @@
           <t>2x Spektrum 5Ah 100c 4S LiPo batteries (vs. Minotaur) MaxAmps 9000XL 6S LiPo batteries (vs. DUCK!) 2x GensAce 7.5Ah 100c 4S LiPo batteries (vs. Blade and Uppercut) [ 2 ]</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
           <t>Piranha</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -22461,16 +22158,11 @@
           <t>Electric Ray</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>World Championship IV (Withdrew)</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>Team Robot Revolution</t>
@@ -22496,12 +22188,6 @@
           <t>Ribbot (Lucas Buermeyer)</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -22514,7 +22200,6 @@
           <t>2x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22530,7 +22215,6 @@
           <t>BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>Bots FC</t>
@@ -22551,17 +22235,11 @@
           <t>Vertical spinner</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
           <t>Shatter! Bliss 2 Doomba and Friends</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -22574,7 +22252,6 @@
           <t>4x 6374-192kV Motors</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22625,15 +22302,11 @@
           <t>2x 1.8Ah MaxAmps batteries</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
           <t>Krusty Grab</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -22646,7 +22319,6 @@
           <t>2x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22662,7 +22334,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>Quicksilver Robotics</t>
@@ -22688,12 +22359,6 @@
           <t>Gruff (John Flaacke IV)</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -22706,7 +22371,6 @@
           <t>2x Magmotors (NPC Charity Open-2009 Collegiate Championship)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>250lbs (WC IV) 120lbs (NPC Charity Open-2009 Collegiate Championship)</t>
@@ -22717,7 +22381,6 @@
           <t>World Championship I (Not selected) World Championship IV</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Falconizer (NPC Charity Open)</t>
@@ -22743,7 +22406,6 @@
           <t>Twin drum spinners (WC IV) Single drum spinner (NPC Charity Open-2009 Collegiate Championship)</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr">
         <is>
           <t>MaxAmps LiPo batteries</t>
@@ -22759,7 +22421,6 @@
           <t>Hydra , Fusion , Red Square , Son of Whyachi , Warrior , Warrior Clan , Whyachi , Why Not , Y-Pout , YU812 , Falcon15 , Buzzkill</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr">
         <is>
           <t>Collegiate Championship 2009</t>
@@ -22782,7 +22443,6 @@
           <t>4x TD6374 Motors</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>203lbs</t>
@@ -22793,8 +22453,6 @@
           <t>World Championship IV</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>Team Danby</t>
@@ -22825,15 +22483,11 @@
           <t>4.5Ah 25C Nanotech LiPo batteries</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr">
         <is>
           <t>Predator , Slammo! , Apex</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -22841,8 +22495,6 @@
           <t>Free Shipping</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>250lbs (WC III-WC VI) 210lbs (WC VII-Present) [ 1 ]</t>
@@ -22858,7 +22510,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2019) BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>Team Special Delivery</t>
@@ -22884,7 +22535,6 @@
           <t>Voltronic , The Swarm (Stephen Felk) Lucky , Wipe Out #2 (Gary Gin) Yeti (James Arluck, Ange Santaguida) VD6.0 , Wrecks , Shockwave (James Arluck) Robo Master (Jim Yeh, Forrest Yeh) Agent X (Jim Yeh)</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs</t>
@@ -22895,9 +22545,6 @@
           <t>The Big B</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -22910,7 +22557,6 @@
           <t>Brushless motors</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -22926,7 +22572,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>Team Whyachi</t>
@@ -22957,15 +22602,11 @@
           <t>18x 4S LiPo batteries</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
           <t>Hydra , Son of Whyachi , Whyachi , YU812 , Y-Pout , Why Not , Red Square , Warrior , Warrior Clan , Falcon , Warrior SKF , Falcon15 , 1A , 3A . POW , BABS , Ricochet , Buzzkill</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -22973,9 +22614,6 @@
           <t>GRABOT</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>World Championship V</t>
@@ -23011,13 +22649,6 @@
           <t>Grabbing arms Wedge</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -23025,8 +22656,6 @@
           <t>Gamma 9</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -23037,7 +22666,6 @@
           <t>World Championship III World Championship V</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>Gamma 9 from Outer Space (WC V)</t>
@@ -23068,16 +22696,11 @@
           <t>BattleSaw (Curtis Nemeth)</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
           <t>Namreko 3000 , Gammatron , Gammacide</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -23090,7 +22713,6 @@
           <t>4x AmpFlow motors (2x per half)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>250lbs (125lbs each)</t>
@@ -23136,12 +22758,6 @@
           <t>Slap Box (Dominic &amp; Hunter Yankauskas) Bolt , MacGuffin , ZAP (Ben Hayton)</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -23154,7 +22770,6 @@
           <t>2x A28-150 AmpFlow motors</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>248lbs</t>
@@ -23170,7 +22785,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>Team Raptor</t>
@@ -23201,15 +22815,11 @@
           <t>8S 5Ah batteries</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr">
         <is>
           <t>Alpha Raptor , Tripulta Raptor , Pack Raptors , Carnage Raptor , W.L.O.W.</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -23222,7 +22832,6 @@
           <t>2x TP5680 brushless motors (WC VII-Present) 2x Short Magmotors (WC III-WC VI)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -23238,7 +22847,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>Robotic Death Company</t>
@@ -23279,9 +22887,6 @@
           <t>Megabyte , Rambite , Invader , Cobalt , Super Megabyte , Agsma</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -23294,7 +22899,6 @@
           <t>4x Scorpion SII-4035-450KV motors</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -23310,7 +22914,6 @@
           <t>BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>Combat Robotics at Berkeley</t>
@@ -23341,15 +22944,11 @@
           <t>10S 6.5Ah LiPo battery (WC VII-BB: Champions II) 8S 8Ah LiPo battery (WC VI-BB: Champions I)</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr">
         <is>
           <t>Holy CR@B , Thunderstorm</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -23362,7 +22961,6 @@
           <t>4x Ampflow E30-400 brushed motors (WC IV)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -23408,12 +23006,6 @@
           <t>Quasar (Sam McAmis) Extinguisher (John Flaacke IV) Slammo! (Jason Rogers)</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -23426,7 +23018,6 @@
           <t>2x Maytech 8085 brushless motors</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -23442,7 +23033,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>Team HUGE</t>
@@ -23473,11 +23063,6 @@
           <t>12x 6S 2.8Ah LiPo batteries [ 1 ]</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -23490,7 +23075,6 @@
           <t>2x Castle 1515 brushless motors</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>242-250lbs</t>
@@ -23551,9 +23135,6 @@
           <t>Skorpios</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -23566,7 +23147,6 @@
           <t>2x TP5680 Brushless inrunner motors</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>225lbs</t>
@@ -23627,9 +23207,6 @@
           <t>Calypso</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -23642,7 +23219,6 @@
           <t>4x Brushless motors</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -23703,9 +23279,6 @@
           <t>Son of Whyachi , Whyachi , YU812 , Y-Pout , Why Not , Red Square , Warrior , Warrior Clan , Fusion , Falcon , Warrior SKF , Falcon15 , 1A , 3A . POW , BABS , Ricochet , Buzzkill</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -23718,7 +23291,6 @@
           <t>2x NeuMotor 8038 motors</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>238-250lbs</t>
@@ -23779,9 +23351,6 @@
           <t>Hot Mess , Vertigo</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -23794,7 +23363,6 @@
           <t>2x AmpFlow 48V motors</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>231½-248lbs</t>
@@ -23805,8 +23373,6 @@
           <t>World Championship III</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Team Toad</t>
@@ -23837,15 +23403,11 @@
           <t>MaxAmps 36V LiPo batteries</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr">
         <is>
           <t>Texas Twister , El Furro , Ice Chip , TadPole , SnowCone , WindChill , IceCube , SnowFlake , IceBerg , FrostBite</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -23858,7 +23420,6 @@
           <t>2x Magmotors</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>250lbs (WC I-Present) 120lbs (2004-2007)</t>
@@ -23909,15 +23470,11 @@
           <t>2x 6S 5Ah LiPo batteries</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr">
         <is>
           <t>Edge , Vault</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -23925,8 +23482,6 @@
           <t>JackPot</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>243-250lbs</t>
@@ -23982,10 +23537,6 @@
           <t>BattleBots Proving Ground (2023) BattleBots FaceOffs (2024) BattleBots Proving Ground (2025) BattleBots FaceOffs (2025)</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -23998,15 +23549,11 @@
           <t>4x Ampflow A28-400 brushed motors [ 1 ] [ 2 ]</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>World Championship IV</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>Tomco Designs</t>
@@ -24032,12 +23579,6 @@
           <t>Radioactive , X/Change (Kevin Cleasby)</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -24045,8 +23586,6 @@
           <t>Jäger</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>246lbs (Combined)</t>
@@ -24057,7 +23596,6 @@
           <t>World Championship V (Withdrew) World Championship VI World Championship VII (Not selected)</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>Jager</t>
@@ -24088,12 +23626,6 @@
           <t>Nelly the Ellybot (Charlie Dangerfield) Big Dill (Andy Russell, Emmanuel Carrillo) Abrasion (Ed Hodges)</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -24106,7 +23638,6 @@
           <t>2x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24117,8 +23648,6 @@
           <t>World Championship IV World Championship V (Withdrew) World Championship VI (Not selected)</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>Team Burntpopcorn</t>
@@ -24139,13 +23668,6 @@
           <t>Horizontal bar spinner</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -24158,7 +23680,6 @@
           <t>4x HyperDrive motors (WC VII-Present) 2x NPC-T74 motors (WC III-BB: Champions I)</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>249lbs</t>
@@ -24199,13 +23720,6 @@
           <t>Crusher Articulating vertical spinner (WC VII-Present)</t>
         </is>
       </c>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -24218,7 +23732,6 @@
           <t>4x Ampflow-A28-250 motors</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24269,15 +23782,11 @@
           <t>17Ah LiFePO batteries (6-8S)</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr">
         <is>
           <t>CU-JAW , Diesector , Tazbot , Easty Beast , Root Canal , Gear Crow</t>
         </is>
       </c>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -24290,7 +23799,6 @@
           <t>2x Magmotors</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24336,7 +23844,6 @@
           <t>Free Shipping , The Big B , Wipe Out #2 (Gary Gin) Captain Shrederator (Zac O'Donnell) Defender , Bite Force , FrostBite , Scrap Metal (Rob Masek) Deep Six , Triton , Malice (Andrew Burghgraef) Witch Doctor , Hack &amp; Slash (Kurtis Wanner) BravePart , PitBot (Mark Demers, Jeff Hayashida, Mohan Gurunathan, Robert Frankovich, Jerome Johnson) Cobalt (Matt Olson, Mark Demers) Nerd Killer , Shockwave , VD6.0 , Wrecks , Yeti (James Arluck)</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
           <t>BattleBots Proving Ground BattleBots FaceOffs</t>
@@ -24347,9 +23854,6 @@
           <t>Ziggy , CycloneBot</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -24362,7 +23866,6 @@
           <t>6x 9kW Brushless motors</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24423,9 +23926,6 @@
           <t>Bad Kitty , CatKong</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -24438,7 +23938,6 @@
           <t>2x S28-D4-400x Long Magmotors</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24454,7 +23953,6 @@
           <t>BattleBots: Bounty Hunters re:MARS all:STARS (2022) BattleBots: Champions I BattleBots: Champions II BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>Team Malice</t>
@@ -24480,16 +23978,11 @@
           <t>Wrecks , Shatter! (Adrian "Bunny" Liaw) Silver Shield (David Liaw) Big Dill (Isaak Malers) Banshee (David Small, David Rush) Drago (Nick Dobrikov) Skorpios (Adrian "Bunny" Liaw, David Liaw, Jonathan LaPlain) Doomba and Friends (Adrian "Bunny" Liaw) Tombstone , Swamp Thing , Darkness , The Raven , Skorpios (Ray Billings) Captain Shrederator (Jonathan LaPlain) Horizon (Peter Garnache) VD6.0 (Alex Tramiel) JackPot (Scott Johnston)</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs (2024)</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -24502,7 +23995,6 @@
           <t>2x RV-100 motors</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24518,7 +24010,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>Team Mammoth</t>
@@ -24549,11 +24040,6 @@
           <t>MaxAmps LiPo batteries</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -24561,8 +24047,6 @@
           <t>Mecha Rampage</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24573,8 +24057,6 @@
           <t>World Championship III</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>C2 Robotics (formerly Team Coolrobots)</t>
@@ -24600,16 +24082,11 @@
           <t>Yeti , Chunk (Christian Carlberg)</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
           <t>OverDrive , Minion , OverKill , Toe-Crusher , Dreadnought , Knee-Breaker , UpperCut , TriDent , Nasty , Little Killer</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -24622,7 +24099,6 @@
           <t>4x Maytech 6374 brushless motors</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>250lbs (WC IV-WC V) 235lbs (WC VI)</t>
@@ -24668,16 +24144,11 @@
           <t>Uppercut (Sarah Pohorecky) Starchild , RIPperoni (Brandon Zalinsky, Sarah Pohorecky)</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
           <t>Parallax , Talos</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr"/>
-      <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -24685,8 +24156,6 @@
           <t>Pain Train</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24702,7 +24171,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>Team Shreddit</t>
@@ -24733,15 +24201,11 @@
           <t>3x 5Ah 45C LiPo batteries</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
           <t>SHREDDIT BRO!</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -24754,7 +24218,6 @@
           <t>2x Long Magmotors</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
           <t>169-230lbs</t>
@@ -24770,7 +24233,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>Team Doom Robotics</t>
@@ -24796,12 +24258,6 @@
           <t>Tombstone , Malice (Ray Billings) Brutality (Alternative identity)</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -24814,7 +24270,6 @@
           <t>4x AmpFlow E30-400 motors</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
           <t>245lbs</t>
@@ -24830,7 +24285,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>Team X</t>
@@ -24851,17 +24305,11 @@
           <t>Vertical spinner</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
           <t>4x Turnigy Nanotech 5Ah 5S LiPo batteries</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
-      <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -24874,7 +24322,6 @@
           <t>2x S28-150 Magmotors</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24890,7 +24337,6 @@
           <t>BattleBots: Champions I BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>Team Ribbot (formerly Team WPI)</t>
@@ -24916,12 +24362,6 @@
           <t>Electric Ray (Lucas Buermeyer)</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
-      <c r="P79" t="inlineStr"/>
-      <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -24929,23 +24369,6 @@
           <t>Rotator</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -24953,8 +24376,6 @@
           <t>Rusty</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -24995,17 +24416,11 @@
           <t>Jackhammer Sledgehammer Lifter</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs (2024)</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -25013,23 +24428,6 @@
           <t>SMEEEEEEEEEEE</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -25042,7 +24440,6 @@
           <t>2x T&amp;P brushless motors 2x Black Max motors (WC III)</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25098,10 +24495,6 @@
           <t>BattleBots: Destruct-A-Thon</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="inlineStr"/>
-      <c r="R83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -25114,7 +24507,6 @@
           <t>2x MC160 motors</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>220lbs</t>
@@ -25160,16 +24552,11 @@
           <t>Deviled Egg , Riptide (Zak Hassanein) P.T. Bruiser , Robot X (Edward Robinson)</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr">
         <is>
           <t>Mantasaur , TriloBot</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -25182,7 +24569,6 @@
           <t>4x Castle 2028 brushless motors</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25233,15 +24619,11 @@
           <t>MaxAmps LiPo batteries</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr">
         <is>
           <t>Emulsifier Doomba and Friends Bliss 2</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -25254,7 +24636,6 @@
           <t>2x Long Magmotors (WC II - WC IV) 4x Short Magmotors (WC V-BB: Champions II) 2x Long Magmotors &amp; 2x Small Magmotors (WCVIII-Present)</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>~250lbs</t>
@@ -25270,7 +24651,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2019) BattleBots: Bounty Hunters re:MARS all:STARS BattleBots Challenge (2022) BattleBots: Champions I BattleBots: Champions II BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>Bot Bash Party Crew (formerly Offbeat Robotics )</t>
@@ -25311,9 +24691,6 @@
           <t>Dragon King</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr"/>
-      <c r="Q86" t="inlineStr"/>
-      <c r="R86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -25321,23 +24698,6 @@
           <t>SlamMow!</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
-      <c r="Q87" t="inlineStr"/>
-      <c r="R87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -25345,8 +24705,6 @@
           <t>Slap Box</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25392,12 +24750,6 @@
           <t>Gemini (Dominic Yankauskas, Hunter Yankauskas)</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
-      <c r="R88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -25410,7 +24762,6 @@
           <t>4x Astro 90 Cobalt motors</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>250lbs (WC I-Present) 315lbs (Season 3.0-5.0)</t>
@@ -25461,7 +24812,6 @@
           <t>Various 4S and 5S LiPo batteries</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr">
         <is>
           <t>Whyachi , YU812 , Y-Pout , Why Not , Red Square , Warrior , Hydra , Fusion , Falcon , Warrior Clan , Warrior SKF , Falcon15 , 1A , 3A . POW , BABS , Ricochet , Buzzkill</t>
@@ -25472,8 +24822,6 @@
           <t>Season 3.0 Season 4.0 Season 5.0</t>
         </is>
       </c>
-      <c r="Q89" t="inlineStr"/>
-      <c r="R89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -25486,7 +24834,6 @@
           <t>4x 6474 Brushless motors</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25502,7 +24849,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>Team PRIDE</t>
@@ -25528,12 +24874,6 @@
           <t>Doomba (Liz Chavarria)</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -25541,8 +24881,6 @@
           <t>SubZero</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>250lbs (WC II-Present) 220lbs (2009 Pro Championship) 140lbs (NPC Charity Open-JavaOne 2007)</t>
@@ -25588,7 +24926,6 @@
           <t>Lock-Jaw (Reginald Wilson, Logan Davis, Brady Davis) The Cone Army , Mixmaster (Alex Horne) Texas Twister (Brady Davis) Mudhole Bullfrog , Total Anarchy (Jon Durand) Switchback (Logan Davis)</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr">
         <is>
           <t>2004 NPC Charity Open R3: Rochester Robot Rampage BattleBots JavaOne 2007</t>
@@ -25599,13 +24936,11 @@
           <t>Team Hammertime Hammertime , Bounty Hunter Team XD Steel Reign , HazMatXD , Adonai , RobotussinDM , ...Tysant</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr"/>
       <c r="Q91" t="inlineStr">
         <is>
           <t>Pro Championship 2009</t>
         </is>
       </c>
-      <c r="R91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -25618,7 +24953,6 @@
           <t>2x TP5680 brushless motors</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>250lbs (WC IV-Present) 235lbs (WC III)</t>
@@ -25634,7 +24968,6 @@
           <t>BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>Seems Reasonable Robotics</t>
@@ -25665,15 +24998,11 @@
           <t>4x 5.4Ah 6S LiPo batteries</t>
         </is>
       </c>
-      <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr">
         <is>
           <t>Blip , The Twins</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -25686,7 +25015,6 @@
           <t>Various Ranglebox motors</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>~250lb combined</t>
@@ -25697,7 +25025,6 @@
           <t>World Championship III World Championship IV</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>Four Horsemen</t>
@@ -25723,21 +25050,16 @@
           <t>Various horizontal spinners</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
           <t>5S LiPo batteries</t>
         </is>
       </c>
-      <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr">
         <is>
           <t>Creepy Crawlies , Bull Dog , Little Sister</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr"/>
-      <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -25750,7 +25072,6 @@
           <t>2x Maytech 8085 brushless outrunners</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>220lbs (Pro Championship 2009) 250lbs (WC I-Present) 340lbs (NPC Charity Open)</t>
@@ -25766,7 +25087,6 @@
           <t>2004 NPC Charity Open re:MARS all:STARS (2019) BattleBots: Bounty Hunters re:MARS all:STARS (2022) BattleBots: Champions I BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>Hardcore Robotics</t>
@@ -25777,7 +25097,6 @@
           <t>Ray Billings (Captain) Rick Russ (WC I-BB: Champions I) Justin Billings Brittney Billings (WC II, WC VI-Present) Lorna West (WC V-BB: Champions I) Susan Billings (WC II) Roy Hellen (WC V-BB: Bounty Hunters) Tyler Nguyen (WC V-BB: Champions I) Kevin Benesi (WC VI-Present) Teri Billings (WC VI-Present) Zach Lytle (BB FaceOffs 2024)</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr">
         <is>
           <t>Horizontal bar spinner</t>
@@ -25803,13 +25122,11 @@
           <t>Darkness , The Raven , Swamp Thing , The Mortician</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr"/>
       <c r="Q94" t="inlineStr">
         <is>
           <t>Pro Championship 2009</t>
         </is>
       </c>
-      <c r="R94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -25817,8 +25134,6 @@
           <t>Tracer</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25834,7 +25149,6 @@
           <t>BattleBots: Bounty Hunters</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>Team KYMERA</t>
@@ -25865,11 +25179,6 @@
           <t>12-13S 20Ah LiPo batteries</t>
         </is>
       </c>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
-      <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -25877,8 +25186,6 @@
           <t>Uppercut</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25894,7 +25201,6 @@
           <t>BattleBots: Champions I</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
           <t>Team Uppercut (formerly MIT Combat Robotics Club)</t>
@@ -25920,12 +25226,6 @@
           <t>SawBlaze (Alex Hattori) Road Rash (Jared DiCarlo, Alex Hattori) P1 (Sarah Pohorecky) Starchild , Ripperoni (Anna Zolnikov, Sarah Pohorecky, Austin Brown) The Dentist (Austin Brown) LOLcano , Deathicator (Austin Brown, Anna Zolnikov)</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
-      <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -25933,8 +25233,6 @@
           <t>Valkyrie</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -25950,7 +25248,6 @@
           <t>BattleBots: Bounty Hunters BattleBots: Champions I BattleBots: Champions II BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>Team VALKYRIE (WC VI-Present) Team Questionable Designs (WC III-WC V)</t>
@@ -25976,16 +25273,11 @@
           <t>SawBlaze (Lucy Du, John Mayo) , RIPperoni , Starchild , Road Rash (Frederick Moore) Overhaul (Lucy Du) Whiplash , Defender , Splatter , Think Tank (Jason Vasquez)</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs (2024)</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr"/>
-      <c r="P97" t="inlineStr"/>
-      <c r="Q97" t="inlineStr"/>
-      <c r="R97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -25998,7 +25290,6 @@
           <t>2x Mini Magmotors (WC IV-Present) 2x 48v AmpFlow motors (WC III)</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>250lbs</t>
@@ -26014,7 +25305,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2019) re:MARS all:STARS BattleBots Challenge (2022) BattleBots: Champions I BattleBots: Champions II</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>Team Fast Electric Robots</t>
@@ -26040,16 +25330,11 @@
           <t>VD6.0 (Jeff Vasquez) Manta (Matt Vasquez)</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr">
         <is>
           <t>Deb Bot , Matts Bammer , Think Tank , Splatter , Defender</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr"/>
-      <c r="Q98" t="inlineStr"/>
-      <c r="R98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -26062,7 +25347,6 @@
           <t>2x Long Magmotors</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>250lbs (WC I-Present) 120lbs (BotsIQ 2010-BotsIQ 2011)</t>
@@ -26078,7 +25362,6 @@
           <t>re:MARS all:STARS BattleBots Challenge (2019) BattleBots: Bounty Hunters BattleBots: Champions I BattleBots Pro League (2026)</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>Team Witch Doctor (formerly Busted Nuts Robotics)</t>
@@ -26104,19 +25387,1570 @@
           <t>Lucky , Hack &amp; Slash (Kurtis Wanner) Mohawk (Christian Chiriboga) Coincidence , Brutus , Overhaul (Adam Bercu) Safety Factor , Category 5 (Andrea Suarez, Mike Gellatly) The Kerminator , Marvinator , Commander K-9 (Andrea Gellatly, Carolina de Freitas) UM Spin EM (Andrea Suarez)</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr">
         <is>
           <t>BattleBots FaceOffs (2024)</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr"/>
-      <c r="P99" t="inlineStr"/>
-      <c r="Q99" t="inlineStr"/>
       <c r="R99" t="inlineStr">
         <is>
           <t>BotsIQ 2010 BotsIQ 2011</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Robot_Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Avg_Win_Pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Overall_Avg_Win_Pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Lift</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Small_Sample_Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2x S28-400 Magmotors (9hp) [ 2 ]</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.408</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2x Maytech 6880 brushless motors (WC VII-Present) 2x 48v Bosch DC motors (WC I-BB: Bounty Hunters) 2x 36V Magmotor S28-200 motors (Season 5.0)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.064</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>6x 9kW Brushless motors</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.006</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4x Brushless motors</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.765</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2x Maytech MTO6365 motors (BB Pro League 2026)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4x Brushless TP Motors</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2x TP5680 brushless motors</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.663</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2x Long Magmotors (WC II - WC IV) 4x Short Magmotors (WC V-BB: Champions II) 2x Long Magmotors &amp; 2x Small Magmotors (WCVIII-Present)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2x Maytech 8085 brushless motors</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2x Mini Magmotors (WC IV-Present) 2x 48v AmpFlow motors (WC III)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2x RV-100 motors</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2x S28-150 Magmotors</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2x S28-D4-400x Long Magmotors</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2x T&amp;P brushless motors 2x Black Max motors (WC III)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>4x Castle 2028 brushless motors</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.606</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2x 8025 Brushless motors (WCVIII-Present) 2x Magmotors (WC IV-BB: Champions II)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>4x Ampflow-A28-250 motors</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.481</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2x HyperDrive motors</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.404</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>4x 6374-192kV Motors</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.375</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2x Magmotors</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.355</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2x Castle 1515 brushless motors</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.204</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>4x Long Magmotors</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.204</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>4x RV-120E brushless motors</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.204</v>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>6x 3" Brushed motors (WC II) 4x motors (WC I</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.204</v>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Various Ranglebox motors</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.204</v>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>WC III-Present)</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.204</v>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>4x Maytech 6374 brushless motors</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.148</v>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2x NeuMotor 8038 motors</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.142</v>
+      </c>
+      <c r="G29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2x TP5680 brushless motors (WC VII-Present) 2x Short Magmotors (WC III-WC VI)</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.142</v>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>4x Scorpion SII-4035-450KV motors</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="G31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2x Brushless motors (WC III) 2x NPC brushed motors (WC II)</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="G32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Brushless motors</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="G33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>4x Maytech 65162 brushless motors</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="G34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>4x Magmotors</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="G35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2x Long Magmotors (WC VII-Present) 2x NPC-T64 motors (WC VI)</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="G36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2x Magmotors (NPC Charity Open-2009 Collegiate Championship)</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="G37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2x Maytech 8085 brushless outrunners</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="G38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>4x AmpFlow motors (2x per half)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="G39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>4x Ampflow E30-400 brushed motors (WC IV)</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+      <c r="G40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2x Castle 2028 brushless motors</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="G41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2x AmpFlow 48V motors</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="G42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2x Long Magmotors</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="G43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2x TP5680 Brushless inrunner motors</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="G44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>4x Flipsky 6384 brushless motors</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="G45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>T-MOTOR P80III KV100 motors</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.602</v>
+      </c>
+      <c r="G46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2x A28-150 AmpFlow motors</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="G47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>4x HyperDrive motors (WC VII-Present) 2x NPC-T74 motors (WC III-BB: Champions I)</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="G48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2x Custom motors</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2x Electric scooter motors</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2x MC160 motors</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2x Surpass 70120 brushless motors</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>4x 6474 Brushless motors</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>4x Ampflow A28-400 brushed motors [ 1 ] [ 2 ]</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>4x TD6374 Motors</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>4x AmpFlow E30-400 motors</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>4x Astro 90 Cobalt motors</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement code changes to enhance functionality and improve performance
</commit_message>
<xml_diff>
--- a/battlebots_2015_2025.xlsx
+++ b/battlebots_2015_2025.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season 12 (2022)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weapons_BattleBotsCom" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot_Features" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Correlations" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40737,6 +40738,3994 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G148"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Robot_Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Avg_Win_Pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Overall_Avg_Win_Pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Lift</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Small_Sample_Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2x S28-400 Magmotors (9hp) [ 2 ]</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.525</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2x Short brushless Magmotors</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.259</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2x Maytech 6880 brushless motors (WC VII-Present) 2x 48v Bosch DC motors (WC I-BB: Bounty Hunters) 2x 36V Magmotor S28-200 motors (Season 5.0)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.156</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2x Maytech 8085 brushless outrunners</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.021</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4x Brushless motors</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.932</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2x Maytech MTO6365 motors (BB Pro League 2026)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.882</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4x Brushless TP Motors</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.882</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4x Brushed LEM motors</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.845</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2x Mini Magmotors (WC IV-Present) 2x 48v AmpFlow motors (WC III)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.797</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2x Maytech 8085 brushless motors</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.758</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2x T&amp;P brushless motors 2x Black Max motors (WC III)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.718</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2x 8025 Brushless motors (WCVIII-Present) 2x Magmotors (WC IV-BB: Champions II)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.647</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4x Astro 90 Cobalt motors</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.621</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6x 9kW Brushless motors</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.621</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>6x 3" Brushed motors (WC II) 4x motors (WC I</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>WC III-Present)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2x TP5680 brushless motors</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.607</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2x 1415 Aveox 3-turn brushless DC motors</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.581</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2x S28-150 Magmotors</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.581</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2x S28-D4-400x Long Magmotors</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.581</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2x Long Magmotors (WC II - WC IV) 4x Short Magmotors (WC V-BB: Champions II) 2x Long Magmotors &amp; 2x Small Magmotors (WCVIII-Present)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.579</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.526</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2x HyperDrive motors</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>4x 6374-192kV Motors</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4x Castle 2028 brushless motors</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>4x Ampflow-A28-250 motors</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.494</v>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2x NPC-T64 brushed motors</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.405</v>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2x Magmotors</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.395</v>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2x Brushless motors (WC III) 2x NPC brushed motors (WC II)</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2x Castle 1515 brushless motors</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2x Custom brushless motors</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2x NeuMotor 8038 motors</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2x RV-100 motors</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2x Short Magmotors (2009-WC III) 2x 12hp Briggs &amp; Stratton motors (Season 5.0) [ 1 ]</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>4x Long Magmotors</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>4x RV-120E brushless motors</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ampflow motors</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2x TP5680 brushless motors (WC VII-Present) 2x Short Magmotors (WC III-WC VI)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.249</v>
+      </c>
+      <c r="G38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>4x Magmotors</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.432</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1.139</v>
+      </c>
+      <c r="G39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>4x Scorpion SII-4035-450KV motors</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="G40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2x Long Magmotors</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>7</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.401</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.058</v>
+      </c>
+      <c r="G41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Brushless motors</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>4x Maytech 6374 brushless motors</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.393</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.036</v>
+      </c>
+      <c r="G43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>4x Maytech 65162 brushless motors</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="G44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2x Maytech 6374 Brushless motors</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="G45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2x A28-150 AmpFlow motors</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="G46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2x Long Magmotor brushed motors</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2x Long Magmotors (WC VII-Present) 2x NPC-T64 motors (WC VI)</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2x Magmotors (NPC Charity Open-2009 Collegiate Championship)</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>4x AmpFlow motors (2x per half)</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>4x Brushed motors</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Pittman DC brushed motors (Comedy Central)</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Various Ranglebox motors</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2x Castle 2028 brushless motors</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>7</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="G54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>4x Ampflow E30-400 brushed motors (WC IV)</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="G55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2x AmpFlow 48V motors</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2x Ampflow A40-300 motors</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2x NPC T64 motors</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G58" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2x TP5680 Brushless inrunner motors</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>3x Maytech 6396 brushless motors</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>4x Flipsky 6384 brushless motors</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>T-MOTOR P80III KV100 motors</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2x 80mm brushless outrunner motors (WC V-Present) 2x Sk3-6374 motors (WC I-WC III)</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="G63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>4x HyperDrive motors (WC VII-Present) 2x NPC-T74 motors (WC III-BB: Champions I)</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>4x TD6374 Motors</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="G65" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2x 528-150 Magmotors</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2x Ampflow A28-400 motors</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2x Custom motors</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2x Electric scooter motors</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2x MC160 motors</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2x S28-400 Motors (WC V-BB: Champions I) 2x Neumotors (WC VII-BB: Champions II) 4x Castle brushless motors (BB Proving Ground-Present)</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2x Short Magmotors</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2x Surpass 70120 brushless motors</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>3x Flipsky 6384 190Kv motors (Drive) 3x unnamed 360Kv motors (Steering)</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>3x Maytech brushless motors</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>4x 6474 Brushless motors</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>4x AmpFlow E30-400 motors</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>4x AmpFlow F30-150 brushed motors</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>4x Ampflow A28-150G brushed motors</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>4x Ampflow A28-400 brushed motors [ 1 ] [ 2 ]</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>4x Bosch GPA-750 motors (Season 4.0) 4x Dustin Motors (Season 5.0)</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>4x NPC brushed motors</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Ampflow A28-150 motor (Rear leg</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>WC I-WC II) Castle brushless motors (BB Proving Ground)</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>WC I-WC II) Motenergy ME0909 motor (Vertical spinner</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2x AmpFlow A28-400-F48 motors</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2x Ampflow A28-150 motors</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2x Ampflow brushed motors</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2x Ampflow motors</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2x Bosch GPA-24-750 motors</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>4x SK3 motors</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Drive_Type</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Etek motors</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Lifter + Vertical Disk Spinner</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F93" t="n">
+        <v>2.635</v>
+      </c>
+      <c r="G93" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Articulated Lifter</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F94" t="n">
+        <v>1.797</v>
+      </c>
+      <c r="G94" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Vertical Disc Spinner</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1.797</v>
+      </c>
+      <c r="G95" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Launcher</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0.672</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1.771</v>
+      </c>
+      <c r="G96" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Egg Beater Spinner</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>3</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F97" t="n">
+        <v>1.679</v>
+      </c>
+      <c r="G97" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Hammer Saw</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>2</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="E98" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F98" t="n">
+        <v>1.622</v>
+      </c>
+      <c r="G98" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Crusher</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>2</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F99" t="n">
+        <v>1.581</v>
+      </c>
+      <c r="G99" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Horizontal Drum Spinner</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1.581</v>
+      </c>
+      <c r="G100" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Puncher</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0.596</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F101" t="n">
+        <v>1.571</v>
+      </c>
+      <c r="G101" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Bar spinner (vertical)</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>7</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0.587</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F102" t="n">
+        <v>1.546</v>
+      </c>
+      <c r="G102" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Sword</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="E103" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F103" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="G103" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Bar spinner (horizontal)</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>15</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F104" t="n">
+        <v>1.428</v>
+      </c>
+      <c r="G104" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Articulated Drum Spinner</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F105" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G105" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Beater</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G106" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Drum Spinner</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G107" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Grappler Saw</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G108" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Rotary Flipper</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F109" t="n">
+        <v>1.318</v>
+      </c>
+      <c r="G109" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Disc spinner (vertical)</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>15</v>
+      </c>
+      <c r="D110" t="n">
+        <v>0.491</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F110" t="n">
+        <v>1.293</v>
+      </c>
+      <c r="G110" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Full Body Spinner</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F111" t="n">
+        <v>1.249</v>
+      </c>
+      <c r="G111" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Modular</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>2</v>
+      </c>
+      <c r="D112" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F112" t="n">
+        <v>1.202</v>
+      </c>
+      <c r="G112" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Flipper</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>5</v>
+      </c>
+      <c r="D113" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F113" t="n">
+        <v>1.156</v>
+      </c>
+      <c r="G113" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Drum spinner</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>10</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0.406</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F114" t="n">
+        <v>1.069</v>
+      </c>
+      <c r="G114" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Disc spinner (horizontal)</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>7</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0.401</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F115" t="n">
+        <v>1.057</v>
+      </c>
+      <c r="G115" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Horizontal Disc combo</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F116" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G116" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Swiss Army Bot- flipper</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>1</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F117" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G117" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Vertical Drum</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>1</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F118" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G118" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
+      </c>
+      <c r="D119" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F119" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G119" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>horizontal spinner</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F120" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G120" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>kitchen sink</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F121" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G121" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>vertical spinner</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F122" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="G122" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Fowl Language</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F123" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="G123" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Kinetic Ring Spinning Flipper</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G124" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Pneumatic hammer</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G125" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Undercutter + Lifter</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G126" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>flamethrower</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G127" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>launcher</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G128" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>vertical bar spinner</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="G129" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>6</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="G130" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Power Hammer</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.822</v>
+      </c>
+      <c r="G131" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Grappler + Torch</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="G132" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Grappler</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>7</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G133" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Lifter</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>10</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="G134" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Axe</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G135" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Horizontal Hammersaw</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="G136" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Kinetic Krusher</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Full Bodied Spinner</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>2</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="G138" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Full Bodied Drum Spinner</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="G139" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Ring Spinner</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>2</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="G140" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Fire Attack Piercer</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Multibot</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Multiple Weapons</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Poker</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Shooter</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Teeth (Spinning)</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Thwackbot</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Weapon_Type</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Articulated Bar Spinner (vertical)</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>